<commit_message>
Drop redundant date_mid; correction sheet shows matiere_auto
date_mid was exactly round((start+end)/2) in 100% of rows in both
languages, so it is stored as start/end only and derived at load in
01-networks. Verified A/B on identical data: graphs, matiere
distributions, Heldendichtung counts and median dates all unchanged.

The correction sheet's reference column is renamed matiere_auto and
holds the *automatic* resolution rather than the corrected value. It
previously held the corrected one, so matiere == override on all 26
French rows and the sheet looked like a no-op. Replaying step 9 from
the algorithmic export now measurably applies 26 corrections:
France 146->147, Britain 59->62, Rome 47->44, Other 42->53,
Unknown 13->7, England 6->0.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/french_works_EdB.xlsx
+++ b/data/french_works_EdB.xlsx
@@ -451,7 +451,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>matiere</t>
+          <t>matiere_auto</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Rome</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Rome</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Rome</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Rome</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Rome</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Rome</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Britain</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>England</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>England</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>England</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>England</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>England</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>France</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Britain</t>
+          <t>Rome</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Britain</t>
+          <t>Rome</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rome</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rome</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Britain</t>
+          <t>Rome</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -2719,7 +2719,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Britain</t>
+          <t>Rome</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>England</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -3959,7 +3959,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Britain</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Britain</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
@@ -4399,7 +4399,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Rome</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Britain</t>
+          <t>Rome</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -5143,7 +5143,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Rome</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Britain</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">

</xml_diff>